<commit_message>
local file updates and added in colab notebooks
</commit_message>
<xml_diff>
--- a/data/Infra-FM-timing-log.xlsx
+++ b/data/Infra-FM-timing-log.xlsx
@@ -14,10 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="23">
-  <si>
-    <t/>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="22">
   <si>
     <t>starting file size (KB)</t>
   </si>
@@ -144,64 +141,61 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="19">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
+      <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -508,296 +502,318 @@
   <dimension ref="A1:O8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="16" width="15.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="17" width="19.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="17" width="15.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="14" width="15.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="15" width="19.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="16" width="15.576428571428572" customWidth="1" bestFit="1"/>
     <col min="4" max="4" style="17" width="51.005" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="16" width="45.86214285714286" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="16" width="34.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="16" width="35.57642857142857" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="16" width="26.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="16" width="21.005" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="15" width="45.86214285714286" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="15" width="34.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="15" width="35.57642857142857" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="15" width="26.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="15" width="21.005" customWidth="1" bestFit="1"/>
     <col min="10" max="10" style="18" width="29.433571428571426" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="16" width="25.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="14" width="25.433571428571426" customWidth="1" bestFit="1"/>
     <col min="12" max="12" style="18" width="29.433571428571426" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="19" width="30.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="19" width="38.71928571428572" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="18" width="30.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="18" width="38.71928571428572" customWidth="1" bestFit="1"/>
     <col min="15" max="15" style="18" width="19.433571428571426" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="1"/>
+      <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="I1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="J1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="K1" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="L1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="M1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="N1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="O1" s="1" t="s">
         <v>13</v>
-      </c>
-      <c r="O1" s="2" t="s">
-        <v>14</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
-      <c r="A2" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B2" s="5">
+      <c r="A2" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="6">
         <v>18437659</v>
       </c>
-      <c r="C2" s="6">
+      <c r="C2" s="7">
         <v>12682.8</v>
       </c>
-      <c r="D2" s="6">
+      <c r="D2" s="7">
         <v>12412800</v>
       </c>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="4"/>
       <c r="J2" s="7"/>
-      <c r="K2" s="3"/>
+      <c r="K2" s="5"/>
       <c r="L2" s="7"/>
-      <c r="M2" s="8"/>
-      <c r="N2" s="8"/>
+      <c r="M2" s="6"/>
+      <c r="N2" s="6"/>
       <c r="O2" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" s="6">
+        <v>33349492</v>
+      </c>
+      <c r="C3" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="5">
-        <v>33349492</v>
-      </c>
-      <c r="C3" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="D3" s="6">
+      <c r="D3" s="7">
         <v>20771611</v>
       </c>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
-      <c r="I3" s="3"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
       <c r="J3" s="7"/>
-      <c r="K3" s="3"/>
+      <c r="K3" s="5"/>
       <c r="L3" s="7"/>
-      <c r="M3" s="8"/>
-      <c r="N3" s="8"/>
+      <c r="M3" s="6"/>
+      <c r="N3" s="6"/>
       <c r="O3" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
-      <c r="A4" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B4" s="5">
+      <c r="A4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="6">
         <v>751228</v>
       </c>
-      <c r="C4" s="6">
+      <c r="C4" s="7">
         <v>459.5</v>
       </c>
-      <c r="D4" s="6">
+      <c r="D4" s="7">
         <v>512504</v>
       </c>
-      <c r="E4" s="10">
+      <c r="E4" s="9">
         <v>439.8</v>
       </c>
-      <c r="F4" s="11">
+      <c r="F4" s="10">
         <v>71</v>
       </c>
-      <c r="G4" s="11">
+      <c r="G4" s="10">
         <v>116</v>
       </c>
-      <c r="H4" s="11">
+      <c r="H4" s="10">
         <v>1917</v>
       </c>
-      <c r="I4" s="11">
+      <c r="I4" s="10">
         <v>1807</v>
       </c>
-      <c r="J4" s="12" t="s">
-        <v>0</v>
-      </c>
-      <c r="K4" s="3"/>
-      <c r="L4" s="12" t="s">
-        <v>0</v>
-      </c>
-      <c r="M4" s="13" t="s">
-        <v>0</v>
-      </c>
-      <c r="N4" s="14"/>
-      <c r="O4" s="15"/>
+      <c r="J4" s="1"/>
+      <c r="K4" s="5"/>
+      <c r="L4" s="1"/>
+      <c r="M4" s="1"/>
+      <c r="N4" s="11"/>
+      <c r="O4" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
-      <c r="A5" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="B5" s="5">
+      <c r="A5" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" s="6">
         <v>15380515</v>
       </c>
-      <c r="C5" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="D5" s="6">
+      <c r="C5" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="7">
         <v>10619855</v>
       </c>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
-      <c r="I5" s="3"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4"/>
+      <c r="G5" s="4"/>
+      <c r="H5" s="4"/>
+      <c r="I5" s="4"/>
       <c r="J5" s="7"/>
-      <c r="K5" s="3"/>
+      <c r="K5" s="5"/>
       <c r="L5" s="7"/>
-      <c r="M5" s="8"/>
-      <c r="N5" s="8"/>
+      <c r="M5" s="6"/>
+      <c r="N5" s="6"/>
       <c r="O5" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
-      <c r="A6" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B6" s="5">
+      <c r="A6" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" s="6">
         <v>1480999</v>
       </c>
-      <c r="C6" s="6">
+      <c r="C6" s="7">
         <v>779.9</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="7">
         <v>1043780</v>
       </c>
-      <c r="E6" s="10">
+      <c r="E6" s="9">
         <v>771.5</v>
       </c>
-      <c r="F6" s="11">
+      <c r="F6" s="10">
         <v>216</v>
       </c>
-      <c r="G6" s="11">
+      <c r="G6" s="10">
         <v>328</v>
       </c>
-      <c r="H6" s="11">
+      <c r="H6" s="10">
         <v>5957</v>
       </c>
-      <c r="I6" s="11">
+      <c r="I6" s="10">
         <v>5583</v>
       </c>
-      <c r="J6" s="12" t="s">
-        <v>0</v>
-      </c>
-      <c r="K6" s="3"/>
-      <c r="L6" s="12" t="s">
-        <v>0</v>
-      </c>
-      <c r="M6" s="13" t="s">
-        <v>0</v>
-      </c>
-      <c r="N6" s="14"/>
-      <c r="O6" s="15"/>
+      <c r="J6" s="3">
+        <v>58.86</v>
+      </c>
+      <c r="K6" s="13">
+        <v>3286</v>
+      </c>
+      <c r="L6" s="3">
+        <v>58.34</v>
+      </c>
+      <c r="M6" s="2">
+        <v>100</v>
+      </c>
+      <c r="N6" s="11">
+        <v>3257</v>
+      </c>
+      <c r="O6" s="12">
+        <v>4816.1</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
-      <c r="A7" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="B7" s="5">
+      <c r="A7" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="6">
         <v>7511059</v>
       </c>
-      <c r="C7" s="6">
+      <c r="C7" s="7">
         <v>5434</v>
       </c>
-      <c r="D7" s="6">
+      <c r="D7" s="7">
         <v>5429796</v>
       </c>
-      <c r="E7" s="10">
+      <c r="E7" s="9">
         <v>5283.2</v>
       </c>
-      <c r="F7" s="11">
+      <c r="F7" s="10">
         <v>382</v>
       </c>
-      <c r="G7" s="11">
+      <c r="G7" s="10">
         <v>505</v>
       </c>
-      <c r="H7" s="11">
+      <c r="H7" s="10">
         <v>11687</v>
       </c>
-      <c r="I7" s="11">
+      <c r="I7" s="10">
         <v>11044</v>
       </c>
-      <c r="J7" s="6"/>
-      <c r="K7" s="3"/>
-      <c r="L7" s="6"/>
-      <c r="M7" s="5"/>
-      <c r="N7" s="5"/>
-      <c r="O7" s="6"/>
+      <c r="J7" s="7">
+        <v>55.52</v>
+      </c>
+      <c r="K7" s="13">
+        <v>6132</v>
+      </c>
+      <c r="L7" s="7">
+        <v>53.14</v>
+      </c>
+      <c r="M7" s="6">
+        <v>100</v>
+      </c>
+      <c r="N7" s="6">
+        <v>5869</v>
+      </c>
+      <c r="O7" s="7">
+        <v>8939</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
-      <c r="A8" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B8" s="5">
+      <c r="A8" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" s="6">
         <v>3832092</v>
       </c>
-      <c r="C8" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="D8" s="6">
+      <c r="C8" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="D8" s="7">
         <v>2723448</v>
       </c>
-      <c r="E8" s="11">
+      <c r="E8" s="10">
         <v>2279</v>
       </c>
-      <c r="F8" s="11">
+      <c r="F8" s="10">
         <v>768</v>
       </c>
-      <c r="G8" s="11">
+      <c r="G8" s="10">
         <v>992</v>
       </c>
-      <c r="H8" s="11">
+      <c r="H8" s="10">
         <v>21240</v>
       </c>
-      <c r="I8" s="11">
+      <c r="I8" s="10">
         <v>17899</v>
       </c>
-      <c r="J8" s="7"/>
-      <c r="K8" s="3"/>
-      <c r="L8" s="7"/>
-      <c r="M8" s="8"/>
-      <c r="N8" s="8"/>
-      <c r="O8" s="7"/>
+      <c r="J8" s="7">
+        <v>63.86</v>
+      </c>
+      <c r="K8" s="13">
+        <v>11431</v>
+      </c>
+      <c r="L8" s="7">
+        <v>63.2</v>
+      </c>
+      <c r="M8" s="6">
+        <v>100</v>
+      </c>
+      <c r="N8" s="6">
+        <v>11313</v>
+      </c>
+      <c r="O8" s="7">
+        <v>14389.9</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
europe substations and fetching modifications
</commit_message>
<xml_diff>
--- a/data/Infra-FM-timing-log.xlsx
+++ b/data/Infra-FM-timing-log.xlsx
@@ -87,7 +87,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -104,12 +104,6 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -141,7 +135,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="14">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -152,49 +146,34 @@
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -502,24 +481,24 @@
   <dimension ref="A1:O8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="14" width="15.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="15" width="19.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="16" width="15.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="17" width="51.005" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="15" width="45.86214285714286" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="15" width="34.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="15" width="35.57642857142857" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="15" width="26.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="15" width="21.005" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="18" width="29.433571428571426" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="14" width="25.433571428571426" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="18" width="29.433571428571426" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="18" width="30.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="18" width="38.71928571428572" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="18" width="19.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="10" width="15.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="11" width="19.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="12" width="15.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="13" width="51.005" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="11" width="45.86214285714286" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="11" width="34.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="11" width="35.57642857142857" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="11" width="26.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="11" width="21.005" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="13" width="29.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="11" width="25.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="13" width="29.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="11" width="30.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="11" width="38.71928571428572" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="13" width="19.433571428571426" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -545,22 +524,22 @@
       <c r="I1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="K1" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" s="3" t="s">
         <v>13</v>
       </c>
     </row>
@@ -568,13 +547,13 @@
       <c r="A2" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B2" s="6">
+      <c r="B2" s="4">
         <v>18437659</v>
       </c>
-      <c r="C2" s="7">
+      <c r="C2" s="6">
         <v>12682.8</v>
       </c>
-      <c r="D2" s="7">
+      <c r="D2" s="6">
         <v>12412800</v>
       </c>
       <c r="E2" s="4"/>
@@ -582,130 +561,174 @@
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
-      <c r="J2" s="7"/>
-      <c r="K2" s="5"/>
-      <c r="L2" s="7"/>
-      <c r="M2" s="6"/>
-      <c r="N2" s="6"/>
-      <c r="O2" s="7"/>
+      <c r="J2" s="6"/>
+      <c r="K2" s="4"/>
+      <c r="L2" s="6"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
+      <c r="O2" s="6"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
       <c r="A3" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B3" s="6">
+      <c r="B3" s="4">
         <v>33349492</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="7">
+      <c r="D3" s="6">
         <v>20771611</v>
       </c>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
-      <c r="H3" s="4"/>
-      <c r="I3" s="4"/>
-      <c r="J3" s="7"/>
-      <c r="K3" s="5"/>
-      <c r="L3" s="7"/>
-      <c r="M3" s="6"/>
-      <c r="N3" s="6"/>
-      <c r="O3" s="7"/>
+      <c r="E3" s="4">
+        <v>19130</v>
+      </c>
+      <c r="F3" s="4">
+        <v>15930</v>
+      </c>
+      <c r="G3" s="4">
+        <v>22526</v>
+      </c>
+      <c r="H3" s="4">
+        <v>592997</v>
+      </c>
+      <c r="I3" s="4">
+        <v>505951</v>
+      </c>
+      <c r="J3" s="6"/>
+      <c r="K3" s="4"/>
+      <c r="L3" s="6"/>
+      <c r="M3" s="4"/>
+      <c r="N3" s="4"/>
+      <c r="O3" s="6"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
       <c r="A4" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="6">
+      <c r="B4" s="4">
         <v>751228</v>
       </c>
-      <c r="C4" s="7">
+      <c r="C4" s="6">
         <v>459.5</v>
       </c>
-      <c r="D4" s="7">
+      <c r="D4" s="6">
         <v>512504</v>
       </c>
-      <c r="E4" s="9">
+      <c r="E4" s="6">
         <v>439.8</v>
       </c>
-      <c r="F4" s="10">
+      <c r="F4" s="4">
         <v>71</v>
       </c>
-      <c r="G4" s="10">
+      <c r="G4" s="4">
         <v>116</v>
       </c>
-      <c r="H4" s="10">
+      <c r="H4" s="4">
         <v>1917</v>
       </c>
-      <c r="I4" s="10">
+      <c r="I4" s="4">
         <v>1807</v>
       </c>
-      <c r="J4" s="1"/>
-      <c r="K4" s="5"/>
-      <c r="L4" s="1"/>
-      <c r="M4" s="1"/>
-      <c r="N4" s="11"/>
-      <c r="O4" s="12"/>
+      <c r="J4" s="3">
+        <v>76.37</v>
+      </c>
+      <c r="K4" s="4">
+        <v>1380</v>
+      </c>
+      <c r="L4" s="3">
+        <v>98.62</v>
+      </c>
+      <c r="M4" s="2">
+        <v>100</v>
+      </c>
+      <c r="N4" s="8">
+        <v>1361</v>
+      </c>
+      <c r="O4" s="9">
+        <v>3266.2</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
       <c r="A5" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="6">
+      <c r="B5" s="4">
         <v>15380515</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="D5" s="7">
+      <c r="D5" s="6">
         <v>10619855</v>
       </c>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="4"/>
-      <c r="J5" s="7"/>
-      <c r="K5" s="5"/>
-      <c r="L5" s="7"/>
-      <c r="M5" s="6"/>
-      <c r="N5" s="6"/>
-      <c r="O5" s="7"/>
+      <c r="E5" s="4">
+        <v>11486.9</v>
+      </c>
+      <c r="F5" s="4">
+        <v>4342</v>
+      </c>
+      <c r="G5" s="4">
+        <v>5738</v>
+      </c>
+      <c r="H5" s="4">
+        <v>137929</v>
+      </c>
+      <c r="I5" s="4">
+        <v>127244</v>
+      </c>
+      <c r="J5" s="6">
+        <v>14.72</v>
+      </c>
+      <c r="K5" s="4">
+        <v>18730</v>
+      </c>
+      <c r="L5" s="6">
+        <v>14.49</v>
+      </c>
+      <c r="M5" s="4">
+        <v>100</v>
+      </c>
+      <c r="N5" s="4">
+        <v>18441</v>
+      </c>
+      <c r="O5" s="6">
+        <v>79459.9</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
       <c r="A6" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="6">
+      <c r="B6" s="4">
         <v>1480999</v>
       </c>
-      <c r="C6" s="7">
+      <c r="C6" s="6">
         <v>779.9</v>
       </c>
-      <c r="D6" s="7">
+      <c r="D6" s="6">
         <v>1043780</v>
       </c>
-      <c r="E6" s="9">
+      <c r="E6" s="6">
         <v>771.5</v>
       </c>
-      <c r="F6" s="10">
+      <c r="F6" s="4">
         <v>216</v>
       </c>
-      <c r="G6" s="10">
+      <c r="G6" s="4">
         <v>328</v>
       </c>
-      <c r="H6" s="10">
+      <c r="H6" s="4">
         <v>5957</v>
       </c>
-      <c r="I6" s="10">
+      <c r="I6" s="4">
         <v>5583</v>
       </c>
       <c r="J6" s="3">
         <v>58.86</v>
       </c>
-      <c r="K6" s="13">
+      <c r="K6" s="4">
         <v>3286</v>
       </c>
       <c r="L6" s="3">
@@ -714,10 +737,10 @@
       <c r="M6" s="2">
         <v>100</v>
       </c>
-      <c r="N6" s="11">
+      <c r="N6" s="8">
         <v>3257</v>
       </c>
-      <c r="O6" s="12">
+      <c r="O6" s="9">
         <v>4816.1</v>
       </c>
     </row>
@@ -725,46 +748,46 @@
       <c r="A7" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B7" s="6">
+      <c r="B7" s="4">
         <v>7511059</v>
       </c>
-      <c r="C7" s="7">
+      <c r="C7" s="6">
         <v>5434</v>
       </c>
-      <c r="D7" s="7">
+      <c r="D7" s="6">
         <v>5429796</v>
       </c>
-      <c r="E7" s="9">
+      <c r="E7" s="6">
         <v>5283.2</v>
       </c>
-      <c r="F7" s="10">
+      <c r="F7" s="4">
         <v>382</v>
       </c>
-      <c r="G7" s="10">
+      <c r="G7" s="4">
         <v>505</v>
       </c>
-      <c r="H7" s="10">
+      <c r="H7" s="4">
         <v>11687</v>
       </c>
-      <c r="I7" s="10">
+      <c r="I7" s="4">
         <v>11044</v>
       </c>
-      <c r="J7" s="7">
+      <c r="J7" s="6">
         <v>55.52</v>
       </c>
-      <c r="K7" s="13">
+      <c r="K7" s="4">
         <v>6132</v>
       </c>
-      <c r="L7" s="7">
+      <c r="L7" s="6">
         <v>53.14</v>
       </c>
-      <c r="M7" s="6">
+      <c r="M7" s="4">
         <v>100</v>
       </c>
-      <c r="N7" s="6">
+      <c r="N7" s="4">
         <v>5869</v>
       </c>
-      <c r="O7" s="7">
+      <c r="O7" s="6">
         <v>8939</v>
       </c>
     </row>
@@ -772,46 +795,46 @@
       <c r="A8" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="6">
+      <c r="B8" s="4">
         <v>3832092</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D8" s="7">
+      <c r="D8" s="6">
         <v>2723448</v>
       </c>
-      <c r="E8" s="10">
+      <c r="E8" s="4">
         <v>2279</v>
       </c>
-      <c r="F8" s="10">
+      <c r="F8" s="4">
         <v>768</v>
       </c>
-      <c r="G8" s="10">
+      <c r="G8" s="4">
         <v>992</v>
       </c>
-      <c r="H8" s="10">
+      <c r="H8" s="4">
         <v>21240</v>
       </c>
-      <c r="I8" s="10">
+      <c r="I8" s="4">
         <v>17899</v>
       </c>
-      <c r="J8" s="7">
+      <c r="J8" s="6">
         <v>63.86</v>
       </c>
-      <c r="K8" s="13">
+      <c r="K8" s="4">
         <v>11431</v>
       </c>
-      <c r="L8" s="7">
+      <c r="L8" s="6">
         <v>63.2</v>
       </c>
-      <c r="M8" s="6">
+      <c r="M8" s="4">
         <v>100</v>
       </c>
-      <c r="N8" s="6">
+      <c r="N8" s="4">
         <v>11313</v>
       </c>
-      <c r="O8" s="7">
+      <c r="O8" s="6">
         <v>14389.9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
recent changes - updated sampling of substations for high vol continents
</commit_message>
<xml_diff>
--- a/data/Infra-FM-timing-log.xlsx
+++ b/data/Infra-FM-timing-log.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="23">
   <si>
     <t>starting file size (KB)</t>
   </si>
@@ -38,6 +38,9 @@
   </si>
   <si>
     <t>num assets after dedup</t>
+  </si>
+  <si>
+    <t>num assets used in PC fetch</t>
   </si>
   <si>
     <t>PC Percent of accepted tiles (%)</t>
@@ -135,7 +138,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -154,6 +157,9 @@
     </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
     </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -478,24 +484,25 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:O8"/>
+  <dimension ref="A1:P8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="10" width="15.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="11" width="19.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="12" width="15.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="13" width="51.005" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="11" width="45.86214285714286" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="11" width="34.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="11" width="35.57642857142857" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="11" width="26.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="11" width="21.005" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="13" width="29.433571428571426" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="11" width="25.433571428571426" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="13" width="29.433571428571426" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="11" width="30.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="11" width="38.71928571428572" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="13" width="19.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="11" width="15.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="12" width="19.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="13" width="15.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="14" width="51.005" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="12" width="45.86214285714286" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="12" width="34.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="12" width="35.57642857142857" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="12" width="26.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="12" width="21.005" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="14" width="29.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="12" width="25.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="14" width="29.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="12" width="30.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="12" width="38.71928571428572" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="14" width="19.433571428571426" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
@@ -524,28 +531,31 @@
       <c r="I1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="K1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="L1" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M1" s="3" t="s">
         <v>11</v>
       </c>
       <c r="N1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="O1" s="2" t="s">
         <v>13</v>
+      </c>
+      <c r="P1" s="3" t="s">
+        <v>14</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B2" s="4">
         <v>18437659</v>
@@ -561,22 +571,25 @@
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
-      <c r="J2" s="6"/>
-      <c r="K2" s="4"/>
-      <c r="L2" s="6"/>
-      <c r="M2" s="4"/>
+      <c r="J2" s="7">
+        <v>25000</v>
+      </c>
+      <c r="K2" s="6"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="6"/>
       <c r="N2" s="4"/>
-      <c r="O2" s="6"/>
+      <c r="O2" s="4"/>
+      <c r="P2" s="6"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
       <c r="A3" s="5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B3" s="4">
         <v>33349492</v>
       </c>
-      <c r="C3" s="7" t="s">
-        <v>16</v>
+      <c r="C3" s="8" t="s">
+        <v>17</v>
       </c>
       <c r="D3" s="6">
         <v>20771611</v>
@@ -596,16 +609,19 @@
       <c r="I3" s="4">
         <v>505951</v>
       </c>
-      <c r="J3" s="6"/>
-      <c r="K3" s="4"/>
-      <c r="L3" s="6"/>
-      <c r="M3" s="4"/>
+      <c r="J3" s="7">
+        <v>25000</v>
+      </c>
+      <c r="K3" s="6"/>
+      <c r="L3" s="4"/>
+      <c r="M3" s="6"/>
       <c r="N3" s="4"/>
-      <c r="O3" s="6"/>
+      <c r="O3" s="4"/>
+      <c r="P3" s="6"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
       <c r="A4" s="5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B4" s="4">
         <v>751228</v>
@@ -631,34 +647,37 @@
       <c r="I4" s="4">
         <v>1807</v>
       </c>
-      <c r="J4" s="3">
+      <c r="J4" s="7">
+        <v>1807</v>
+      </c>
+      <c r="K4" s="3">
         <v>76.37</v>
       </c>
-      <c r="K4" s="4">
+      <c r="L4" s="4">
         <v>1380</v>
       </c>
-      <c r="L4" s="3">
+      <c r="M4" s="3">
         <v>98.62</v>
       </c>
-      <c r="M4" s="2">
+      <c r="N4" s="2">
         <v>100</v>
       </c>
-      <c r="N4" s="8">
+      <c r="O4" s="9">
         <v>1361</v>
       </c>
-      <c r="O4" s="9">
+      <c r="P4" s="10">
         <v>3266.2</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
       <c r="A5" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B5" s="4">
         <v>15380515</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D5" s="6">
         <v>10619855</v>
@@ -678,28 +697,31 @@
       <c r="I5" s="4">
         <v>127244</v>
       </c>
-      <c r="J5" s="6">
+      <c r="J5" s="7">
+        <v>25000</v>
+      </c>
+      <c r="K5" s="6">
         <v>14.72</v>
       </c>
-      <c r="K5" s="4">
+      <c r="L5" s="4">
         <v>18730</v>
       </c>
-      <c r="L5" s="6">
+      <c r="M5" s="6">
         <v>14.49</v>
       </c>
-      <c r="M5" s="4">
+      <c r="N5" s="4">
         <v>100</v>
       </c>
-      <c r="N5" s="4">
+      <c r="O5" s="4">
         <v>18441</v>
       </c>
-      <c r="O5" s="6">
+      <c r="P5" s="6">
         <v>79459.9</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
       <c r="A6" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B6" s="4">
         <v>1480999</v>
@@ -725,28 +747,31 @@
       <c r="I6" s="4">
         <v>5583</v>
       </c>
-      <c r="J6" s="3">
+      <c r="J6" s="7">
+        <v>5583</v>
+      </c>
+      <c r="K6" s="3">
         <v>58.86</v>
       </c>
-      <c r="K6" s="4">
+      <c r="L6" s="4">
         <v>3286</v>
       </c>
-      <c r="L6" s="3">
+      <c r="M6" s="3">
         <v>58.34</v>
       </c>
-      <c r="M6" s="2">
+      <c r="N6" s="2">
         <v>100</v>
       </c>
-      <c r="N6" s="8">
+      <c r="O6" s="9">
         <v>3257</v>
       </c>
-      <c r="O6" s="9">
+      <c r="P6" s="10">
         <v>4816.1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
       <c r="A7" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B7" s="4">
         <v>7511059</v>
@@ -772,34 +797,37 @@
       <c r="I7" s="4">
         <v>11044</v>
       </c>
-      <c r="J7" s="6">
+      <c r="J7" s="7">
+        <v>11044</v>
+      </c>
+      <c r="K7" s="6">
         <v>55.52</v>
       </c>
-      <c r="K7" s="4">
+      <c r="L7" s="4">
         <v>6132</v>
       </c>
-      <c r="L7" s="6">
+      <c r="M7" s="6">
         <v>53.14</v>
       </c>
-      <c r="M7" s="4">
+      <c r="N7" s="4">
         <v>100</v>
       </c>
-      <c r="N7" s="4">
+      <c r="O7" s="4">
         <v>5869</v>
       </c>
-      <c r="O7" s="6">
+      <c r="P7" s="6">
         <v>8939</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
       <c r="A8" s="5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B8" s="4">
         <v>3832092</v>
       </c>
-      <c r="C8" s="7" t="s">
-        <v>16</v>
+      <c r="C8" s="8" t="s">
+        <v>17</v>
       </c>
       <c r="D8" s="6">
         <v>2723448</v>
@@ -819,22 +847,25 @@
       <c r="I8" s="4">
         <v>17899</v>
       </c>
-      <c r="J8" s="6">
+      <c r="J8" s="7">
+        <v>17899</v>
+      </c>
+      <c r="K8" s="6">
         <v>63.86</v>
       </c>
-      <c r="K8" s="4">
+      <c r="L8" s="4">
         <v>11431</v>
       </c>
-      <c r="L8" s="6">
+      <c r="M8" s="6">
         <v>63.2</v>
       </c>
-      <c r="M8" s="4">
+      <c r="N8" s="4">
         <v>100</v>
       </c>
-      <c r="N8" s="4">
+      <c r="O8" s="4">
         <v>11313</v>
       </c>
-      <c r="O8" s="6">
+      <c r="P8" s="6">
         <v>14389.9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
removed redundant/legacy files to streamline codebase
</commit_message>
<xml_diff>
--- a/data/Infra-FM-timing-log.xlsx
+++ b/data/Infra-FM-timing-log.xlsx
@@ -93,7 +93,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -110,12 +110,6 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -147,7 +141,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -159,9 +153,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -496,22 +487,22 @@
   <dimension ref="A1:P8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="11" width="15.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="12" width="19.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="13" width="15.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="14" width="51.005" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="12" width="45.86214285714286" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="12" width="34.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="12" width="35.57642857142857" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="12" width="26.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="12" width="21.005" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="12" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="14" width="29.433571428571426" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="12" width="25.433571428571426" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="14" width="29.433571428571426" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="12" width="30.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="12" width="38.71928571428572" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="14" width="19.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="10" width="15.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="11" width="19.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="12" width="15.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="13" width="51.005" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="11" width="45.86214285714286" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="11" width="34.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="11" width="35.57642857142857" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="11" width="26.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="11" width="21.005" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="13" width="29.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="11" width="25.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="13" width="29.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="11" width="30.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="11" width="38.71928571428572" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="13" width="19.433571428571426" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
@@ -540,7 +531,7 @@
       <c r="I1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="J1" s="4" t="s">
         <v>8</v>
       </c>
       <c r="K1" s="3" t="s">
@@ -563,16 +554,16 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="5" t="s">
         <v>15</v>
       </c>
       <c r="B2" s="4">
         <v>18437659</v>
       </c>
-      <c r="C2" s="7">
+      <c r="C2" s="6">
         <v>12682.8</v>
       </c>
-      <c r="D2" s="7">
+      <c r="D2" s="6">
         <v>12412800</v>
       </c>
       <c r="E2" s="4">
@@ -593,24 +584,36 @@
       <c r="J2" s="4">
         <v>25000</v>
       </c>
-      <c r="K2" s="7"/>
-      <c r="L2" s="4"/>
-      <c r="M2" s="7"/>
-      <c r="N2" s="4"/>
-      <c r="O2" s="4"/>
-      <c r="P2" s="7"/>
+      <c r="K2" s="6">
+        <v>99.9</v>
+      </c>
+      <c r="L2" s="4">
+        <v>24974</v>
+      </c>
+      <c r="M2" s="6">
+        <v>98.74</v>
+      </c>
+      <c r="N2" s="4">
+        <v>100</v>
+      </c>
+      <c r="O2" s="4">
+        <v>24659</v>
+      </c>
+      <c r="P2" s="6">
+        <v>25895.9</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="5" t="s">
         <v>16</v>
       </c>
       <c r="B3" s="4">
         <v>33349492</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="7">
+      <c r="D3" s="6">
         <v>20771611</v>
       </c>
       <c r="E3" s="4">
@@ -631,13 +634,13 @@
       <c r="J3" s="4">
         <v>25000</v>
       </c>
-      <c r="K3" s="7">
+      <c r="K3" s="6">
         <v>93.04</v>
       </c>
       <c r="L3" s="4">
         <v>23260</v>
       </c>
-      <c r="M3" s="7">
+      <c r="M3" s="6">
         <v>70.48</v>
       </c>
       <c r="N3" s="4">
@@ -646,24 +649,24 @@
       <c r="O3" s="4">
         <v>17622</v>
       </c>
-      <c r="P3" s="7" t="s">
+      <c r="P3" s="6" t="s">
         <v>18</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="5" t="s">
         <v>19</v>
       </c>
       <c r="B4" s="4">
         <v>751228</v>
       </c>
-      <c r="C4" s="7">
+      <c r="C4" s="6">
         <v>459.5</v>
       </c>
-      <c r="D4" s="7">
+      <c r="D4" s="6">
         <v>512504</v>
       </c>
-      <c r="E4" s="7">
+      <c r="E4" s="6">
         <v>439.8</v>
       </c>
       <c r="F4" s="4">
@@ -693,24 +696,24 @@
       <c r="N4" s="2">
         <v>100</v>
       </c>
-      <c r="O4" s="9">
+      <c r="O4" s="8">
         <v>1361</v>
       </c>
-      <c r="P4" s="10">
+      <c r="P4" s="9">
         <v>3266.2</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="5" t="s">
         <v>20</v>
       </c>
       <c r="B5" s="4">
         <v>15380515</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="D5" s="7">
+      <c r="D5" s="6">
         <v>10619855</v>
       </c>
       <c r="E5" s="4">
@@ -731,13 +734,13 @@
       <c r="J5" s="4">
         <v>127244</v>
       </c>
-      <c r="K5" s="7">
+      <c r="K5" s="6">
         <v>14.72</v>
       </c>
       <c r="L5" s="4">
         <v>18730</v>
       </c>
-      <c r="M5" s="7">
+      <c r="M5" s="6">
         <v>14.49</v>
       </c>
       <c r="N5" s="4">
@@ -746,24 +749,24 @@
       <c r="O5" s="4">
         <v>18441</v>
       </c>
-      <c r="P5" s="7">
+      <c r="P5" s="6">
         <v>79459.9</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="5" t="s">
         <v>21</v>
       </c>
       <c r="B6" s="4">
         <v>1480999</v>
       </c>
-      <c r="C6" s="7">
+      <c r="C6" s="6">
         <v>779.9</v>
       </c>
-      <c r="D6" s="7">
+      <c r="D6" s="6">
         <v>1043780</v>
       </c>
-      <c r="E6" s="7">
+      <c r="E6" s="6">
         <v>771.5</v>
       </c>
       <c r="F6" s="4">
@@ -793,27 +796,27 @@
       <c r="N6" s="2">
         <v>100</v>
       </c>
-      <c r="O6" s="9">
+      <c r="O6" s="8">
         <v>3257</v>
       </c>
-      <c r="P6" s="10">
+      <c r="P6" s="9">
         <v>4816.1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="5" t="s">
         <v>22</v>
       </c>
       <c r="B7" s="4">
         <v>7511059</v>
       </c>
-      <c r="C7" s="7">
+      <c r="C7" s="6">
         <v>5434</v>
       </c>
-      <c r="D7" s="7">
+      <c r="D7" s="6">
         <v>5429796</v>
       </c>
-      <c r="E7" s="7">
+      <c r="E7" s="6">
         <v>5283.2</v>
       </c>
       <c r="F7" s="4">
@@ -831,13 +834,13 @@
       <c r="J7" s="4">
         <v>11044</v>
       </c>
-      <c r="K7" s="7">
+      <c r="K7" s="6">
         <v>55.52</v>
       </c>
       <c r="L7" s="4">
         <v>6132</v>
       </c>
-      <c r="M7" s="7">
+      <c r="M7" s="6">
         <v>53.14</v>
       </c>
       <c r="N7" s="4">
@@ -846,21 +849,21 @@
       <c r="O7" s="4">
         <v>5869</v>
       </c>
-      <c r="P7" s="7">
+      <c r="P7" s="6">
         <v>8939</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
-      <c r="A8" s="6" t="s">
+      <c r="A8" s="5" t="s">
         <v>23</v>
       </c>
       <c r="B8" s="4">
         <v>3832092</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="7">
+      <c r="D8" s="6">
         <v>2723448</v>
       </c>
       <c r="E8" s="4">
@@ -881,13 +884,13 @@
       <c r="J8" s="4">
         <v>17899</v>
       </c>
-      <c r="K8" s="7">
+      <c r="K8" s="6">
         <v>63.86</v>
       </c>
       <c r="L8" s="4">
         <v>11431</v>
       </c>
-      <c r="M8" s="7">
+      <c r="M8" s="6">
         <v>63.2</v>
       </c>
       <c r="N8" s="4">
@@ -896,7 +899,7 @@
       <c r="O8" s="4">
         <v>11313</v>
       </c>
-      <c r="P8" s="7">
+      <c r="P8" s="6">
         <v>14389.9</v>
       </c>
     </row>

</xml_diff>